<commit_message>
Corrected empirical bootstrap values heterochrony analysis to take into account finite number of bootstrap resamples
</commit_message>
<xml_diff>
--- a/output/supplemental_tables/TablesS4-S8.xlsx
+++ b/output/supplemental_tables/TablesS4-S8.xlsx
@@ -294,7 +294,7 @@
     <tableColumn id="6" name="Bootstrap_SE"/>
     <tableColumn id="7" name="CI_95_lower"/>
     <tableColumn id="8" name="CI_95_upper"/>
-    <tableColumn id="9" name="Empirical_P"/>
+    <tableColumn id="9" name="Centred_bootstrap_P"/>
     <tableColumn id="10" name="Bonferroni_P"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
@@ -2277,13 +2277,13 @@
         <v>13</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.85</v>
+        <v>1.88</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>7.027027027027026</v>
+        <v>6.914893617021277</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>4.1e-09</v>
+        <v>5.1e-09</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -2314,13 +2314,13 @@
         <v>45</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>16.29</v>
+        <v>16.58</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>2.762430939226519</v>
+        <v>2.714113389626056</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>8.3e-09</v>
+        <v>1.3e-08</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
@@ -2351,13 +2351,13 @@
         <v>9</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.42</v>
+        <v>1.45</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>6.338028169014085</v>
+        <v>6.206896551724138</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>3.4e-06</v>
+        <v>4e-06</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -2388,13 +2388,13 @@
         <v>13</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>3.13</v>
+        <v>3.19</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>4.15335463258786</v>
+        <v>4.075235109717869</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>6.3e-06</v>
+        <v>7.700000000000001e-06</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -2425,13 +2425,13 @@
         <v>10</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>5.025125628140704</v>
+        <v>4.926108374384237</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>1.2e-05</v>
+        <v>1.4e-05</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -2462,13 +2462,13 @@
         <v>12</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2.92</v>
+        <v>2.97</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>4.109589041095891</v>
+        <v>4.04040404040404</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1.6e-05</v>
+        <v>1.9e-05</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
@@ -2499,13 +2499,13 @@
         <v>10</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>2.06</v>
+        <v>2.1</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>4.854368932038835</v>
+        <v>4.761904761904762</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>1.7e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -2530,19 +2530,19 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>41</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>16.36</v>
+        <v>16.51</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>2.506112469437653</v>
+        <v>2.483343428225318</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>2.1e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
@@ -2573,13 +2573,13 @@
         <v>9</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.78</v>
+        <v>1.81</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>5.056179775280899</v>
+        <v>4.972375690607735</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>3e-05</v>
+        <v>3.5e-05</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -2610,13 +2610,13 @@
         <v>8</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1.49</v>
+        <v>1.52</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>5.369127516778524</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>5.3e-05</v>
+        <v>6.1e-05</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
@@ -2647,13 +2647,13 @@
         <v>17</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2.92</v>
+        <v>2.97</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>5.821917808219178</v>
+        <v>5.723905723905723</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.0001</v>
+        <v>0.00011</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -2669,32 +2669,32 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>GO:0019674</t>
+          <t>GO:0006575</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NAD metabolic process</t>
+          <t>modified amino acid metabolic process</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>1.64</v>
+        <v>3.48</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>4.878048780487805</v>
+        <v>3.448275862068966</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>0.00011</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0005899;N13.HOG0006174;N13.HOG0006298;N13.HOG0006518;N13.HOG0006806;N13.HOG0008484</t>
+          <t>N13.HOG0003437;N13.HOG0004891;N13.HOG0004983;N13.HOG0005767;N13.HOG0005902;N13.HOG0006012;N13.HOG0006180;N13.HOG0006699;N13.HOG0006706;N13.HOG0008012;N13.HOG0009118;N13.HOG0011999</t>
         </is>
       </c>
     </row>
@@ -2706,32 +2706,32 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GO:0006575</t>
+          <t>GO:0019674</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>modified amino acid metabolic process</t>
+          <t>NAD metabolic process</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>3.49</v>
+        <v>1.67</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>3.438395415472779</v>
+        <v>4.790419161676647</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.00011</v>
+        <v>0.00013</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0003437;N13.HOG0004891;N13.HOG0004983;N13.HOG0005767;N13.HOG0005902;N13.HOG0006012;N13.HOG0006180;N13.HOG0006699;N13.HOG0006706;N13.HOG0008012;N13.HOG0009118;N13.HOG0011999</t>
+          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0005899;N13.HOG0006174;N13.HOG0006298;N13.HOG0006518;N13.HOG0006806;N13.HOG0008484</t>
         </is>
       </c>
     </row>
@@ -2743,32 +2743,32 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>GO:0034404</t>
+          <t>GO:0170040</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>nucleobase-containing small molecule biosynthetic process</t>
+          <t>proteinogenic amino acid catabolic process</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>3.98</v>
+        <v>2.1</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>3.266331658291457</v>
+        <v>4.285714285714286</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.00011</v>
+        <v>0.00013</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0004383;N13.HOG0005899;N13.HOG0006063;N13.HOG0006174;N13.HOG0006298;N13.HOG0006468;N13.HOG0006518;N13.HOG0007211;N13.HOG0007469;N13.HOG0007840;N13.HOG0008484</t>
+          <t>N13.HOG0001967;N13.HOG0005222;N13.HOG0005438;N13.HOG0005902;N13.HOG0008016;N13.HOG0008139;N13.HOG0008957;N13.HOG0009118;N13.HOG0011003</t>
         </is>
       </c>
     </row>
@@ -2780,32 +2780,32 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GO:0170040</t>
+          <t>GO:0034404</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>proteinogenic amino acid catabolic process</t>
+          <t>nucleobase-containing small molecule biosynthetic process</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>2.06</v>
+        <v>4.06</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>4.368932038834951</v>
+        <v>3.201970443349754</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.00012</v>
+        <v>0.00013</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0001967;N13.HOG0005222;N13.HOG0005438;N13.HOG0005902;N13.HOG0008016;N13.HOG0008139;N13.HOG0008957;N13.HOG0009118;N13.HOG0011003</t>
+          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0004383;N13.HOG0005899;N13.HOG0006063;N13.HOG0006174;N13.HOG0006298;N13.HOG0006468;N13.HOG0006518;N13.HOG0007211;N13.HOG0007469;N13.HOG0007840;N13.HOG0008484</t>
         </is>
       </c>
     </row>
@@ -2826,19 +2826,19 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>33</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>14.23</v>
+        <v>14.41</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>2.319044272663387</v>
+        <v>2.290076335877862</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.00017</v>
+        <v>0.00019</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
@@ -2863,19 +2863,19 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>38</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>10.53</v>
+        <v>10.65</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3.608736942070276</v>
+        <v>3.568075117370892</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.00033</v>
+        <v>0.00037</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -2891,32 +2891,32 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>GO:0009069</t>
+          <t>GO:0046394</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>serine family amino acid metabolic process</t>
+          <t>carboxylic acid biosynthetic process</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>21</v>
+        <v>102</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1.49</v>
+        <v>7.39</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>4.697986577181208</v>
+        <v>3.788903924221922</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.00042</v>
+        <v>0.00046</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0004957;N13.HOG0004983;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
+          <t>N13.HOG0000561;N13.HOG0001742;N13.HOG0001745;N13.HOG0002865;N13.HOG0003382;N13.HOG0003997;N13.HOG0004383;N13.HOG0004957;N13.HOG0004983;N13.HOG0005438;N13.HOG0005767;N13.HOG0005902;N13.HOG0006012;N13.HOG0006063;N13.HOG0006174;N13.HOG0006298;N13.HOG0006699;N13.HOG0006706;N13.HOG0006707;N13.HOG0007450;N13.HOG0007840;N13.HOG0007931;N13.HOG0008395;N13.HOG0008484;N13.HOG0008677;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
         </is>
       </c>
     </row>
@@ -2928,32 +2928,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>GO:0046394</t>
+          <t>GO:0009069</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>carboxylic acid biosynthetic process</t>
+          <t>serine family amino acid metabolic process</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>103</v>
+        <v>21</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>7.33</v>
+        <v>1.52</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>3.819918144611187</v>
+        <v>4.605263157894737</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.00043</v>
+        <v>0.00047</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0000561;N13.HOG0001742;N13.HOG0001745;N13.HOG0002865;N13.HOG0003382;N13.HOG0003997;N13.HOG0004383;N13.HOG0004957;N13.HOG0004983;N13.HOG0005438;N13.HOG0005767;N13.HOG0005902;N13.HOG0006012;N13.HOG0006063;N13.HOG0006174;N13.HOG0006298;N13.HOG0006699;N13.HOG0006706;N13.HOG0006707;N13.HOG0007450;N13.HOG0007840;N13.HOG0007931;N13.HOG0008395;N13.HOG0008484;N13.HOG0008677;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
+          <t>N13.HOG0004957;N13.HOG0004983;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
         </is>
       </c>
     </row>
@@ -2980,13 +2980,13 @@
         <v>9</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>2.42</v>
+        <v>2.46</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3.71900826446281</v>
+        <v>3.658536585365854</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.00044</v>
+        <v>0.0005</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
@@ -3017,13 +3017,13 @@
         <v>10</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2.92</v>
+        <v>2.97</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>3.424657534246575</v>
+        <v>3.367003367003367</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.00044</v>
+        <v>0.0005</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -3054,13 +3054,13 @@
         <v>8</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>4.020100502512562</v>
+        <v>3.94088669950739</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.00053</v>
+        <v>0.00059</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
@@ -3091,13 +3091,13 @@
         <v>20</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>6.47</v>
+        <v>6.59</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>3.091190108191654</v>
+        <v>3.034901365705615</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.00072</v>
+        <v>0.00082</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -3128,13 +3128,13 @@
         <v>9</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>3.333333333333333</v>
+        <v>3.272727272727273</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.00107</v>
+        <v>0.00121</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
@@ -3150,32 +3150,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>GO:1901607</t>
+          <t>GO:0006633</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>alpha-amino acid biosynthetic process</t>
+          <t>fatty acid biosynthetic process</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>2.35</v>
+        <v>2.24</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>3.829787234042553</v>
+        <v>3.571428571428571</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.00134</v>
+        <v>0.00124</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0004383;N13.HOG0004957;N13.HOG0004983;N13.HOG0005902;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
+          <t>N13.HOG0000561;N13.HOG0003382;N13.HOG0006063;N13.HOG0006707;N13.HOG0007450;N13.HOG0007931;N13.HOG0008395;N13.HOG0008677</t>
         </is>
       </c>
     </row>
@@ -3187,32 +3187,32 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>GO:0006633</t>
+          <t>GO:1901607</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>fatty acid biosynthetic process</t>
+          <t>alpha-amino acid biosynthetic process</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>2.28</v>
+        <v>2.39</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>3.508771929824562</v>
+        <v>3.765690376569037</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.00139</v>
+        <v>0.00143</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0000561;N13.HOG0003382;N13.HOG0006063;N13.HOG0006707;N13.HOG0007450;N13.HOG0007931;N13.HOG0008395;N13.HOG0008677</t>
+          <t>N13.HOG0004383;N13.HOG0004957;N13.HOG0004983;N13.HOG0005902;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882;N13.HOG0009118;N13.HOG0011003</t>
         </is>
       </c>
     </row>
@@ -3224,32 +3224,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>GO:0005975</t>
+          <t>GO:0046395</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>carbohydrate metabolic process</t>
+          <t>carboxylic acid catabolic process</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>178</v>
+        <v>83</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>12.66</v>
+        <v>6.01</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>2.606635071090047</v>
+        <v>4.825291181364393</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.00185</v>
+        <v>0.00193</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0001720;N13.HOG0001742;N13.HOG0001745;N13.HOG0002310;N13.HOG0002563;N13.HOG0002709;N13.HOG0002865;N13.HOG0003075;N13.HOG0003614;N13.HOG0005107;N13.HOG0005142;N13.HOG0005461;N13.HOG0005629;N13.HOG0005679;N13.HOG0005716;N13.HOG0005902;N13.HOG0006174;N13.HOG0006298;N13.HOG0006537;N13.HOG0006699;N13.HOG0006722;N13.HOG0006783;N13.HOG0006806;N13.HOG0007383;N13.HOG0007412;N13.HOG0007555;N13.HOG0007592;N13.HOG0007667;N13.HOG0007840;N13.HOG0008012;N13.HOG0008395;N13.HOG0008484;N13.HOG0008818</t>
+          <t>N13.HOG0001745;N13.HOG0001967;N13.HOG0002821;N13.HOG0003614;N13.HOG0004983;N13.HOG0005222;N13.HOG0005438;N13.HOG0005629;N13.HOG0005679;N13.HOG0005902;N13.HOG0006063;N13.HOG0006510;N13.HOG0006706;N13.HOG0006783;N13.HOG0007413;N13.HOG0007450;N13.HOG0007555;N13.HOG0007686;N13.HOG0007797;N13.HOG0007897;N13.HOG0007931;N13.HOG0008016;N13.HOG0008139;N13.HOG0008494;N13.HOG0008677;N13.HOG0008908;N13.HOG0008957;N13.HOG0009118;N13.HOG0011003</t>
         </is>
       </c>
     </row>
@@ -3261,32 +3261,32 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>GO:0015908</t>
+          <t>GO:0032868</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>fatty acid transport</t>
+          <t>response to insulin</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>1.42</v>
+        <v>8.26</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>4.225352112676057</v>
+        <v>1.573849878934625</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.00203</v>
+        <v>0.0022</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0000906;N13.HOG0003838;N13.HOG0004191;N13.HOG0005679;N13.HOG0005902;N13.HOG0007931</t>
+          <t>N13.HOG0002563;N13.HOG0004383;N13.HOG0005558;N13.HOG0005679;N13.HOG0005834;N13.HOG0005902;N13.HOG0006174;N13.HOG0007372;N13.HOG0007797;N13.HOG0007840;N13.HOG0008395;N13.HOG0008762;N13.HOG0010367</t>
         </is>
       </c>
     </row>
@@ -3298,32 +3298,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>GO:0032868</t>
+          <t>GO:0042178</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>response to insulin</t>
+          <t>xenobiotic catabolic process</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>8.109999999999999</v>
+        <v>2.46</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>1.602959309494451</v>
+        <v>3.252032520325203</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.00203</v>
+        <v>0.00236</v>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0002563;N13.HOG0004383;N13.HOG0005558;N13.HOG0005679;N13.HOG0005834;N13.HOG0005902;N13.HOG0006174;N13.HOG0007372;N13.HOG0007797;N13.HOG0007840;N13.HOG0008395;N13.HOG0008762;N13.HOG0010367</t>
+          <t>N13.HOG0001967;N13.HOG0002708;N13.HOG0005107;N13.HOG0005558;N13.HOG0006063;N13.HOG0006699;N13.HOG0007164;N13.HOG0007555</t>
         </is>
       </c>
     </row>
@@ -3335,69 +3335,69 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>GO:0042178</t>
+          <t>GO:0009066</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>xenobiotic catabolic process</t>
+          <t>aspartate family amino acid metabolic process</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>2.42</v>
+        <v>2.1</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>3.305785123966942</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.00211</v>
+        <v>0.00378</v>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0001967;N13.HOG0002708;N13.HOG0005107;N13.HOG0005558;N13.HOG0006063;N13.HOG0006699;N13.HOG0007164;N13.HOG0007555</t>
+          <t>N13.HOG0001967;N13.HOG0004983;N13.HOG0005222;N13.HOG0005902;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Hibernation</t>
+          <t>Nutrient metabolism</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>GO:0008340</t>
+          <t>GO:0170041</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>determination of adult lifespan</t>
+          <t>non-proteinogenic amino acid metabolic process</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>138</v>
+        <v>29</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>9.82</v>
+        <v>2.1</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>2.342158859470469</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>8.3e-05</v>
+        <v>0.00378</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0000906;N13.HOG0002327;N13.HOG0002352;N13.HOG0002573;N13.HOG0002709;N13.HOG0003075;N13.HOG0005169;N13.HOG0005222;N13.HOG0005558;N13.HOG0005679;N13.HOG0006468;N13.HOG0006699;N13.HOG0006805;N13.HOG0007383;N13.HOG0007641;N13.HOG0007797;N13.HOG0008090;N13.HOG0008109;N13.HOG0008121;N13.HOG0008484;N13.HOG0008808;N13.HOG0008908;N13.HOG0009247</t>
+          <t>N13.HOG0001967;N13.HOG0004383;N13.HOG0004983;N13.HOG0005902;N13.HOG0006699;N13.HOG0006706;N13.HOG0008882</t>
         </is>
       </c>
     </row>
@@ -3409,32 +3409,32 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>GO:0010883</t>
+          <t>GO:0008340</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>regulation of lipid storage</t>
+          <t>determination of adult lifespan</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>42</v>
+        <v>138</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>2.99</v>
+        <v>9.99</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>3.678929765886287</v>
+        <v>2.302302302302302</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0.00011</v>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0000342;N13.HOG0003382;N13.HOG0004886;N13.HOG0004934;N13.HOG0005222;N13.HOG0005679;N13.HOG0006290;N13.HOG0006574;N13.HOG0007833;N13.HOG0008852;N13.HOG0008887</t>
+          <t>N13.HOG0000906;N13.HOG0002327;N13.HOG0002352;N13.HOG0002573;N13.HOG0002709;N13.HOG0003075;N13.HOG0005169;N13.HOG0005222;N13.HOG0005558;N13.HOG0005679;N13.HOG0006468;N13.HOG0006699;N13.HOG0006805;N13.HOG0007383;N13.HOG0007641;N13.HOG0007797;N13.HOG0008090;N13.HOG0008109;N13.HOG0008121;N13.HOG0008484;N13.HOG0008808;N13.HOG0008908;N13.HOG0009247</t>
         </is>
       </c>
     </row>
@@ -3446,32 +3446,32 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>GO:0001666</t>
+          <t>GO:0010883</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>response to hypoxia</t>
+          <t>regulation of lipid storage</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>8.539999999999999</v>
+        <v>3.04</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>1.990632318501171</v>
+        <v>3.618421052631579</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.00111</v>
+        <v>0.00013</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0000906;N13.HOG0001742;N13.HOG0002474;N13.HOG0002563;N13.HOG0002821;N13.HOG0002833;N13.HOG0005169;N13.HOG0005558;N13.HOG0005679;N13.HOG0006106;N13.HOG0006706;N13.HOG0007037;N13.HOG0008395;N13.HOG0009311;N13.HOG0009420;N13.HOG0010084;N13.HOG0011999</t>
+          <t>N13.HOG0000342;N13.HOG0003382;N13.HOG0004886;N13.HOG0004934;N13.HOG0005222;N13.HOG0005679;N13.HOG0006290;N13.HOG0006574;N13.HOG0007833;N13.HOG0008852;N13.HOG0008887</t>
         </is>
       </c>
     </row>
@@ -3483,32 +3483,32 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>GO:0036503</t>
+          <t>GO:0001666</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ERAD pathway</t>
+          <t>response to hypoxia</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>2.42</v>
+        <v>8.69</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>3.305785123966942</v>
+        <v>1.956271576524741</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.00211</v>
+        <v>0.0013</v>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0003332;N13.HOG0005899;N13.HOG0006381;N13.HOG0007010;N13.HOG0008814;N13.HOG0008828;N13.HOG0008844;N13.HOG0011108</t>
+          <t>N13.HOG0000906;N13.HOG0001742;N13.HOG0002474;N13.HOG0002563;N13.HOG0002821;N13.HOG0002833;N13.HOG0005169;N13.HOG0005558;N13.HOG0005679;N13.HOG0006106;N13.HOG0006706;N13.HOG0007037;N13.HOG0008395;N13.HOG0009311;N13.HOG0009420;N13.HOG0010084;N13.HOG0011999</t>
         </is>
       </c>
     </row>
@@ -3520,69 +3520,69 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>GO:0006979</t>
+          <t>GO:0036503</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>response to oxidative stress</t>
+          <t>ERAD pathway</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>11.95</v>
+        <v>2.46</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>1.757322175732218</v>
+        <v>3.252032520325203</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.00245</v>
+        <v>0.00236</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0000906;N13.HOG0001720;N13.HOG0001742;N13.HOG0002708;N13.HOG0004879;N13.HOG0005558;N13.HOG0005679;N13.HOG0005834;N13.HOG0006510;N13.HOG0006805;N13.HOG0007037;N13.HOG0007383;N13.HOG0008012;N13.HOG0008215;N13.HOG0008395;N13.HOG0008511;N13.HOG0008818;N13.HOG0009311;N13.HOG0009420;N13.HOG0009669;N13.HOG0009810</t>
+          <t>N13.HOG0003332;N13.HOG0005899;N13.HOG0006381;N13.HOG0007010;N13.HOG0008814;N13.HOG0008828;N13.HOG0008844;N13.HOG0011108</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Reproduction</t>
+          <t>Hibernation</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>GO:0071364</t>
+          <t>GO:0006979</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>cellular response to epidermal growth factor stimulus</t>
+          <t>response to oxidative stress</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>20</v>
+        <v>168</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>1.42</v>
+        <v>12.17</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>4.225352112676057</v>
+        <v>1.725554642563681</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.00203</v>
+        <v>0.00281</v>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002352;N13.HOG0004383;N13.HOG0005679;N13.HOG0010084;N13.HOG0011272;N13.HOG0011999</t>
+          <t>N13.HOG0000906;N13.HOG0001720;N13.HOG0001742;N13.HOG0002708;N13.HOG0004879;N13.HOG0005558;N13.HOG0005679;N13.HOG0005834;N13.HOG0006510;N13.HOG0006805;N13.HOG0007037;N13.HOG0007383;N13.HOG0008012;N13.HOG0008215;N13.HOG0008395;N13.HOG0008511;N13.HOG0008818;N13.HOG0009311;N13.HOG0009420;N13.HOG0009669;N13.HOG0009810</t>
         </is>
       </c>
     </row>
@@ -3594,32 +3594,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>GO:0008585</t>
+          <t>GO:0071364</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>female gonad development</t>
+          <t>cellular response to epidermal growth factor stimulus</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2.7</v>
+        <v>1.45</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>2.592592592592593</v>
+        <v>4.137931034482759</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.00691</v>
+        <v>0.00222</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0003345;N13.HOG0003347;N13.HOG0006427;N13.HOG0008012;N13.HOG0008968;N13.HOG0009652;N13.HOG0011999</t>
+          <t>N13.HOG0002352;N13.HOG0004383;N13.HOG0005679;N13.HOG0010084;N13.HOG0011272;N13.HOG0011999</t>
         </is>
       </c>
     </row>
@@ -3631,69 +3631,69 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>GO:0016333</t>
+          <t>GO:0008585</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>morphogenesis of follicular epithelium</t>
+          <t>female gonad development</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>1.99</v>
+        <v>2.75</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>3.015075376884422</v>
+        <v>2.545454545454545</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01219</v>
+        <v>0.00745</v>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002495;N13.HOG0003324;N13.HOG0005834;N13.HOG0007833;N13.HOG0008502;N13.HOG0010849</t>
+          <t>N13.HOG0003345;N13.HOG0003347;N13.HOG0006427;N13.HOG0008012;N13.HOG0008968;N13.HOG0009652;N13.HOG0011999</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Reproduction</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>GO:0051262</t>
+          <t>GO:0016333</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>protein tetramerization</t>
+          <t>morphogenesis of follicular epithelium</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2.56</v>
+        <v>2.03</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>5.46875</v>
+        <v>2.955665024630542</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>5.7e-08</v>
+        <v>0.01324</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0002709;N13.HOG0002756;N13.HOG0004055;N13.HOG0004983;N13.HOG0005222;N13.HOG0005558;N13.HOG0006106;N13.HOG0006699;N13.HOG0006880;N13.HOG0006944;N13.HOG0007453;N13.HOG0007897;N13.HOG0008494;N13.HOG0009118</t>
+          <t>N13.HOG0002495;N13.HOG0003324;N13.HOG0005834;N13.HOG0007833;N13.HOG0008502;N13.HOG0010849</t>
         </is>
       </c>
     </row>
@@ -3705,32 +3705,32 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>GO:0051260</t>
+          <t>GO:0051262</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>protein homooligomerization</t>
+          <t>protein tetramerization</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>5.76</v>
+        <v>2.61</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>3.298611111111111</v>
+        <v>5.363984674329502</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>2.3e-06</v>
+        <v>7.1e-08</v>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002352;N13.HOG0002756;N13.HOG0004983;N13.HOG0005169;N13.HOG0005222;N13.HOG0005512;N13.HOG0005558;N13.HOG0005899;N13.HOG0006063;N13.HOG0006415;N13.HOG0006699;N13.HOG0007453;N13.HOG0007897;N13.HOG0008332;N13.HOG0008434;N13.HOG0008494;N13.HOG0009118;N13.HOG0009420;N13.HOG0009571</t>
+          <t>N13.HOG0002709;N13.HOG0002756;N13.HOG0004055;N13.HOG0004983;N13.HOG0005222;N13.HOG0005558;N13.HOG0006106;N13.HOG0006699;N13.HOG0006880;N13.HOG0006944;N13.HOG0007453;N13.HOG0007897;N13.HOG0008494;N13.HOG0009118</t>
         </is>
       </c>
     </row>
@@ -3742,32 +3742,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>GO:0090407</t>
+          <t>GO:0051260</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>organophosphate biosynthetic process</t>
+          <t>protein homooligomerization</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>250</v>
+        <v>81</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>17.79</v>
+        <v>5.87</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>2.304665542439573</v>
+        <v>3.236797274275979</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>3.6e-05</v>
+        <v>3e-06</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0001742;N13.HOG0001745;N13.HOG0002474;N13.HOG0002709;N13.HOG0002865;N13.HOG0003437;N13.HOG0003614;N13.HOG0004055;N13.HOG0004383;N13.HOG0005080;N13.HOG0005461;N13.HOG0005512;N13.HOG0005629;N13.HOG0005767;N13.HOG0005834;N13.HOG0005899;N13.HOG0006063;N13.HOG0006106;N13.HOG0006169;N13.HOG0006174;N13.HOG0006180;N13.HOG0006298;N13.HOG0006495;N13.HOG0006518;N13.HOG0006783;N13.HOG0006806;N13.HOG0006946;N13.HOG0007211;N13.HOG0007450;N13.HOG0007469;N13.HOG0007555;N13.HOG0007575;N13.HOG0007592;N13.HOG0007840;N13.HOG0008012;N13.HOG0008109;N13.HOG0008395;N13.HOG0008454;N13.HOG0008484;N13.HOG0008502;N13.HOG0009118</t>
+          <t>N13.HOG0002352;N13.HOG0002756;N13.HOG0004983;N13.HOG0005169;N13.HOG0005222;N13.HOG0005512;N13.HOG0005558;N13.HOG0005899;N13.HOG0006063;N13.HOG0006415;N13.HOG0006699;N13.HOG0007453;N13.HOG0007897;N13.HOG0008332;N13.HOG0008434;N13.HOG0008494;N13.HOG0009118;N13.HOG0009420;N13.HOG0009571</t>
         </is>
       </c>
     </row>
@@ -3779,32 +3779,32 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>GO:0009100</t>
+          <t>GO:0090407</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>glycoprotein metabolic process</t>
+          <t>organophosphate biosynthetic process</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>106</v>
+        <v>250</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>7.54</v>
+        <v>18.1</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2.387267904509284</v>
+        <v>2.265193370165746</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.00012</v>
+        <v>4.1e-05</v>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0003075;N13.HOG0003332;N13.HOG0003614;N13.HOG0005142;N13.HOG0005899;N13.HOG0006381;N13.HOG0006468;N13.HOG0006495;N13.HOG0007037;N13.HOG0007789;N13.HOG0007833;N13.HOG0008133;N13.HOG0008446;N13.HOG0008679;N13.HOG0008844;N13.HOG0009991;N13.HOG0010849;N13.HOG0011005</t>
+          <t>N13.HOG0001742;N13.HOG0001745;N13.HOG0002474;N13.HOG0002709;N13.HOG0002865;N13.HOG0003437;N13.HOG0003614;N13.HOG0004055;N13.HOG0004383;N13.HOG0005080;N13.HOG0005461;N13.HOG0005512;N13.HOG0005629;N13.HOG0005767;N13.HOG0005834;N13.HOG0005899;N13.HOG0006063;N13.HOG0006106;N13.HOG0006169;N13.HOG0006174;N13.HOG0006180;N13.HOG0006298;N13.HOG0006495;N13.HOG0006518;N13.HOG0006783;N13.HOG0006806;N13.HOG0006946;N13.HOG0007211;N13.HOG0007450;N13.HOG0007469;N13.HOG0007555;N13.HOG0007575;N13.HOG0007592;N13.HOG0007840;N13.HOG0008012;N13.HOG0008109;N13.HOG0008395;N13.HOG0008454;N13.HOG0008484;N13.HOG0008502;N13.HOG0009118</t>
         </is>
       </c>
     </row>
@@ -3816,32 +3816,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>GO:0000381</t>
+          <t>GO:0009100</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>regulation of alternative mRNA splicing, via spliceosome</t>
+          <t>glycoprotein metabolic process</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3.77</v>
+        <v>7.46</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>3.183023872679045</v>
+        <v>2.412868632707775</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0.00025</v>
+        <v>0.00014</v>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0002495;N13.HOG0004087;N13.HOG0004297;N13.HOG0004793;N13.HOG0005049;N13.HOG0006582;N13.HOG0006797;N13.HOG0006880;N13.HOG0008706;N13.HOG0009810;N13.HOG0010314;N13.HOG0010674</t>
+          <t>N13.HOG0003075;N13.HOG0003332;N13.HOG0003614;N13.HOG0005142;N13.HOG0005899;N13.HOG0006381;N13.HOG0006468;N13.HOG0006495;N13.HOG0007037;N13.HOG0007789;N13.HOG0007833;N13.HOG0008133;N13.HOG0008446;N13.HOG0008679;N13.HOG0008844;N13.HOG0009991;N13.HOG0010849;N13.HOG0011005</t>
         </is>
       </c>
     </row>
@@ -3853,32 +3853,32 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>GO:0006406</t>
+          <t>GO:0000381</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>mRNA export from nucleus</t>
+          <t>regulation of alternative mRNA splicing, via spliceosome</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>3.2</v>
+        <v>3.84</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>3.125</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.0009700000000000001</v>
+        <v>0.0003</v>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002495;N13.HOG0004297;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0008706;N13.HOG0008968;N13.HOG0009717</t>
+          <t>N13.HOG0002495;N13.HOG0004087;N13.HOG0004297;N13.HOG0004793;N13.HOG0005049;N13.HOG0006582;N13.HOG0006797;N13.HOG0006880;N13.HOG0008706;N13.HOG0009810;N13.HOG0010314;N13.HOG0010674</t>
         </is>
       </c>
     </row>
@@ -3890,32 +3890,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>GO:0007589</t>
+          <t>GO:0006406</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>body fluid secretion</t>
+          <t>mRNA export from nucleus</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>1.71</v>
+        <v>3.26</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>4.093567251461988</v>
+        <v>3.067484662576687</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.00103</v>
+        <v>0.00111</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0004383;N13.HOG0004886;N13.HOG0005902;N13.HOG0006174;N13.HOG0008215;N13.HOG0010367;N13.HOG0011999</t>
+          <t>N13.HOG0002495;N13.HOG0004297;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0008706;N13.HOG0008968;N13.HOG0009717</t>
         </is>
       </c>
     </row>
@@ -3927,32 +3927,32 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>GO:0031503</t>
+          <t>GO:0007589</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>protein-containing complex localization</t>
+          <t>body fluid secretion</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>111</v>
+        <v>24</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>7.9</v>
+        <v>1.74</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1.89873417721519</v>
+        <v>4.022988505747127</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>0.00104</v>
+        <v>0.00115</v>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002495;N13.HOG0002963;N13.HOG0004297;N13.HOG0005512;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0007592;N13.HOG0008289;N13.HOG0008530;N13.HOG0008706;N13.HOG0008968;N13.HOG0008982</t>
+          <t>N13.HOG0004383;N13.HOG0004886;N13.HOG0005902;N13.HOG0006174;N13.HOG0008215;N13.HOG0010367;N13.HOG0011999</t>
         </is>
       </c>
     </row>
@@ -3964,32 +3964,32 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>GO:0042866</t>
+          <t>GO:0031503</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>pyruvate biosynthetic process</t>
+          <t>protein-containing complex localization</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>1.42</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>4.225352112676057</v>
+        <v>1.865671641791045</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.00203</v>
+        <v>0.00124</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0006174;N13.HOG0006298;N13.HOG0007840;N13.HOG0008484</t>
+          <t>N13.HOG0002495;N13.HOG0002963;N13.HOG0004297;N13.HOG0005512;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0007592;N13.HOG0008289;N13.HOG0008530;N13.HOG0008706;N13.HOG0008968;N13.HOG0008982</t>
         </is>
       </c>
     </row>
@@ -4001,32 +4001,32 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>GO:0071806</t>
+          <t>GO:0042866</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>protein transmembrane transport</t>
+          <t>pyruvate biosynthetic process</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>2.28</v>
+        <v>1.45</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>2.192982456140351</v>
+        <v>4.137931034482759</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>0.00239</v>
+        <v>0.00222</v>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0005679;N13.HOG0006854;N13.HOG0008494;N13.HOG0008536;N13.HOG0011108</t>
+          <t>N13.HOG0001742;N13.HOG0002865;N13.HOG0006174;N13.HOG0006298;N13.HOG0007840;N13.HOG0008484</t>
         </is>
       </c>
     </row>
@@ -4038,32 +4038,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>GO:0006888</t>
+          <t>GO:0071806</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum to Golgi vesicle-mediated transport</t>
+          <t>protein transmembrane transport</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>5.12</v>
+        <v>2.32</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>2.734375</v>
+        <v>2.155172413793104</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.00247</v>
+        <v>0.00256</v>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0003701;N13.HOG0004886;N13.HOG0004934;N13.HOG0005899;N13.HOG0006290;N13.HOG0007757;N13.HOG0007833;N13.HOG0008434;N13.HOG0008852;N13.HOG0008887;N13.HOG0009015;N13.HOG0009137;N13.HOG0009663;N13.HOG0010401</t>
+          <t>N13.HOG0005679;N13.HOG0006854;N13.HOG0008494;N13.HOG0008536;N13.HOG0011108</t>
         </is>
       </c>
     </row>
@@ -4075,32 +4075,32 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>GO:0071166</t>
+          <t>GO:0006606</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>ribonucleoprotein complex localization</t>
+          <t>protein import into nucleus</t>
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>11</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>4.2</v>
+        <v>4.63</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>2.619047619047619</v>
+        <v>2.375809935205184</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>0.0025</v>
+        <v>0.00281</v>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0002495;N13.HOG0004297;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0008530;N13.HOG0008706;N13.HOG0008968;N13.HOG0009717</t>
+          <t>N13.HOG0002963;N13.HOG0005679;N13.HOG0005785;N13.HOG0006291;N13.HOG0007037;N13.HOG0007453;N13.HOG0008289;N13.HOG0008530;N13.HOG0008968;N13.HOG0010401;N13.HOG0011108</t>
         </is>
       </c>
     </row>
@@ -4112,32 +4112,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>GO:0006606</t>
+          <t>GO:0071166</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>protein import into nucleus</t>
+          <t>ribonucleoprotein complex localization</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>11</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>4.55</v>
+        <v>4.27</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>2.417582417582418</v>
+        <v>2.576112412177986</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.00252</v>
+        <v>0.00287</v>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0002963;N13.HOG0005679;N13.HOG0005785;N13.HOG0006291;N13.HOG0007037;N13.HOG0007453;N13.HOG0008289;N13.HOG0008530;N13.HOG0008968;N13.HOG0010401;N13.HOG0011108</t>
+          <t>N13.HOG0002495;N13.HOG0004297;N13.HOG0005785;N13.HOG0006291;N13.HOG0006539;N13.HOG0006797;N13.HOG0007453;N13.HOG0008530;N13.HOG0008706;N13.HOG0008968;N13.HOG0009717</t>
         </is>
       </c>
     </row>
@@ -4164,13 +4164,13 @@
         <v>6</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>1.49</v>
+        <v>1.52</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>4.026845637583893</v>
+        <v>3.947368421052631</v>
       </c>
       <c r="H53" s="7" t="n">
-        <v>0.00268</v>
+        <v>0.00293</v>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
@@ -4442,8 +4442,8 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Empirical_P</t>
+          <t>Centred_bootstrap_P</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -4528,10 +4528,10 @@
         <v>0.02507760409252689</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="J2" s="6" t="n">
-        <v>0.96</v>
+        <v>0.3173652694610778</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -4708,10 +4708,10 @@
         <v>0.01881111009371601</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.008</v>
+        <v>0.1457085828343313</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.048</v>
+        <v>0.874251497005988</v>
       </c>
     </row>
     <row r="8">
@@ -4743,11 +4743,11 @@
       <c r="H8" s="4" t="n">
         <v>0.1354953690114516</v>
       </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>0</v>
+      <c r="I8" s="6" t="n">
+        <v>0.001996007984031936</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.009980039920159681</v>
       </c>
     </row>
     <row r="9">
@@ -4780,7 +4780,7 @@
         <v>0.09013243081129332</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.24</v>
+        <v>0.281437125748503</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>1</v>
@@ -4815,11 +4815,11 @@
       <c r="H10" s="4" t="n">
         <v>0.1140152979234217</v>
       </c>
-      <c r="I10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>0</v>
+      <c r="I10" s="6" t="n">
+        <v>0.001996007984031936</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.009980039920159681</v>
       </c>
     </row>
     <row r="11">
@@ -4852,7 +4852,7 @@
         <v>0.04230563548433951</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.416</v>
+        <v>0.4750499001996008</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>1</v>
@@ -4888,10 +4888,10 @@
         <v>0.031858683321719</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0.04</v>
+        <v>0.03592814371257485</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.2</v>
+        <v>0.1796407185628743</v>
       </c>
     </row>
     <row r="13">
@@ -4923,11 +4923,11 @@
       <c r="H13" s="5" t="n">
         <v>0.1450477999730204</v>
       </c>
-      <c r="I13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>0</v>
+      <c r="I13" s="7" t="n">
+        <v>0.001996007984031936</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>0.007984031936127744</v>
       </c>
     </row>
     <row r="14">
@@ -5032,7 +5032,7 @@
         <v>0.02429753682119604</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.392</v>
+        <v>0.4271457085828343</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1</v>
@@ -5247,11 +5247,11 @@
       <c r="H22" s="4" t="n">
         <v>0.7466977823005572</v>
       </c>
-      <c r="I22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="2" t="n">
-        <v>0</v>
+      <c r="I22" s="6" t="n">
+        <v>0.001996007984031936</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>0.001996007984031936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use fully nested cross-validation for PLS analysis
- Repeat filtering, TMM normalisation, scaling, feature selection and PLS fitting within each training fold
- Update Table S5 and PLS cross-validation outputs
- Add fold-level diagnostics and update analysis metadata, README and reloadable workspaces
</commit_message>
<xml_diff>
--- a/output/supplemental_tables/TablesS4-S8.xlsx
+++ b/output/supplemental_tables/TablesS4-S8.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Leave-one-sample-out season/caste contrasts on PLS axis 1</t>
+          <t>Fully nested leave-one-sample-out season/caste contrasts on PLS axis 1</t>
         </is>
       </c>
     </row>
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>13.83461619573653</v>
+        <v>15.1907835067258</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>3.536009888727905</v>
+        <v>4.067790633172896</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3.912493638617506</v>
+        <v>3.734406432534832</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>0.0001496629912472863</v>
+        <v>0.000285513773193567</v>
       </c>
     </row>
     <row r="3">
@@ -1843,19 +1843,19 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>18.93736448956363</v>
+        <v>20.79307100651</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2.796570013819875</v>
+        <v>3.085264498191223</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>6.771639685750907</v>
+        <v>6.739477610007251</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>4.540423124998843e-10</v>
+        <v>5.33950840770262e-10</v>
       </c>
     </row>
     <row r="4">
@@ -1875,19 +1875,19 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>14.47280065596184</v>
+        <v>15.16962804506235</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3.128278703300059</v>
+        <v>3.423506060033704</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4.62644221587236</v>
+        <v>4.431021233510832</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>9.219636399602757e-06</v>
+        <v>2.037539996101936e-05</v>
       </c>
     </row>
     <row r="5">
@@ -1907,19 +1907,19 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>17.02974035027033</v>
+        <v>18.43619661064062</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2.344355105757014</v>
+        <v>2.712880600678148</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>7.264147103163054</v>
+        <v>6.795800967441052</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>3.649689579496981e-11</v>
+        <v>4.018952358460656e-10</v>
       </c>
     </row>
     <row r="6">
@@ -1939,19 +1939,19 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>11.90068929426988</v>
+        <v>12.71354529300294</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2.83656649839873</v>
+        <v>3.397102959199621</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4.19545577408037</v>
+        <v>3.742466874185742</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>5.1448611974526e-05</v>
+        <v>0.0002774118642823559</v>
       </c>
     </row>
     <row r="7">
@@ -1971,19 +1971,19 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>16.47758073781822</v>
+        <v>18.83256735309037</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>3.399642084053108</v>
+        <v>3.91695192785582</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>4.846857501591279</v>
+        <v>4.807964892078598</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>3.674129061206399e-06</v>
+        <v>4.330032794783674e-06</v>
       </c>
     </row>
     <row r="8">
@@ -2003,19 +2003,19 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>6.325584660043443</v>
+        <v>6.867683979640649</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>3.024912695193412</v>
+        <v>3.468735885853194</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>2.091162720198438</v>
+        <v>1.979880915018535</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.03855482493538535</v>
+        <v>0.04993156740734814</v>
       </c>
     </row>
     <row r="9">
@@ -2035,19 +2035,19 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>11.42833295387055</v>
+        <v>12.46997147942485</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2.278935976381782</v>
+        <v>2.56215751257896</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>5.014767010706053</v>
+        <v>4.866980823077151</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.791382190099256e-06</v>
+        <v>3.373699424199353e-06</v>
       </c>
     </row>
     <row r="10">
@@ -2067,19 +2067,19 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>6.963769120268756</v>
+        <v>6.846528517977203</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>2.640455727663515</v>
+        <v>2.92274034706774</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2.637336065630933</v>
+        <v>2.342503166538906</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.009425585947086</v>
+        <v>0.02074789490369007</v>
       </c>
     </row>
     <row r="11">
@@ -2099,19 +2099,19 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>9.520708814577246</v>
+        <v>10.11309708355547</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>2.441743205182786</v>
+        <v>2.818300253034161</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>3.899144182880828</v>
+        <v>3.58836751785683</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.0001571993880054449</v>
+        <v>0.0004774112019446483</v>
       </c>
     </row>
     <row r="12">
@@ -2131,19 +2131,19 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>4.391657758576801</v>
+        <v>4.390445765917793</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2.329747243862462</v>
+        <v>2.794316963343725</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>124</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.885036142931935</v>
+        <v>1.571205351258403</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.06176535802566898</v>
+        <v>0.1186831866705417</v>
       </c>
     </row>
     <row r="13">
@@ -2163,19 +2163,19 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>8.968549202125134</v>
+        <v>10.50946782600522</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>3.131487270771685</v>
+        <v>3.577878784298491</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>124</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>2.863990310877118</v>
+        <v>2.937345969384424</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.004914163872602449</v>
+        <v>0.003947758446536406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revised Figure 2 & added Figure S4 & fixed mistake in Fig. 3 PNG (missing phylogeny)
</commit_message>
<xml_diff>
--- a/output/supplemental_tables/TablesS4-S8.xlsx
+++ b/output/supplemental_tables/TablesS4-S8.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5A_PLS_axes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5B_PLS_LOOCV" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Fig1_GO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_Fig2A_regressions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_Fig2B_ridge" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_Fig2A_concordance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_Fig2B_HOGs" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table_index'!$A$1:$C$7</definedName>
@@ -21,8 +21,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S5A_PLS_axes'!$A$1:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S5B_PLS_LOOCV'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S6_Fig1_GO'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S7_Fig2A_regressions'!$A$1:$H$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'S8_Fig2B_ridge'!$A$1:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S7_Fig2A_concordance'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'S8_Fig2B_HOGs'!$A$1:$H$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -266,36 +266,35 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SupplementaryTable6" displayName="SupplementaryTable6" ref="A1:H7" headerRowCount="1">
-  <autoFilter ref="A1:H7"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="Stage"/>
-    <tableColumn id="2" name="HOGs"/>
-    <tableColumn id="3" name="Robust_slope"/>
-    <tableColumn id="4" name="SE"/>
-    <tableColumn id="5" name="CI_95_lower"/>
-    <tableColumn id="6" name="CI_95_upper"/>
-    <tableColumn id="7" name="P_value"/>
-    <tableColumn id="8" name="Bonferroni_P"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SupplementaryTable6" displayName="SupplementaryTable6" ref="A1:I37" headerRowCount="1">
+  <autoFilter ref="A1:I37"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Polistes_stage"/>
+    <tableColumn id="2" name="Vespula_stage"/>
+    <tableColumn id="3" name="Jointly_DE_HOGs"/>
+    <tableColumn id="4" name="Concordant_HOGs"/>
+    <tableColumn id="5" name="Concordant_fraction"/>
+    <tableColumn id="6" name="Expected_fraction_from_margins"/>
+    <tableColumn id="7" name="Concordance_log2_odds_ratio"/>
+    <tableColumn id="8" name="One_sided_Fisher_P"/>
+    <tableColumn id="9" name="FDR_P_36_tests"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SupplementaryTable7" displayName="SupplementaryTable7" ref="A1:J22" headerRowCount="1">
-  <autoFilter ref="A1:J22"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Vespula_response_stage"/>
-    <tableColumn id="2" name="Polistes_predictor_stage"/>
-    <tableColumn id="3" name="Stage_lag"/>
-    <tableColumn id="4" name="HOGs"/>
-    <tableColumn id="5" name="Partial_slope"/>
-    <tableColumn id="6" name="Bootstrap_SE"/>
-    <tableColumn id="7" name="CI_95_lower"/>
-    <tableColumn id="8" name="CI_95_upper"/>
-    <tableColumn id="9" name="Centred_bootstrap_P"/>
-    <tableColumn id="10" name="Bonferroni_P"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SupplementaryTable7" displayName="SupplementaryTable7" ref="A1:H15" headerRowCount="1">
+  <autoFilter ref="A1:H15"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="HOG"/>
+    <tableColumn id="2" name="Displayed_gene"/>
+    <tableColumn id="3" name="Functional_group"/>
+    <tableColumn id="4" name="Selected_comparison"/>
+    <tableColumn id="5" name="Polistes L1 late vs early"/>
+    <tableColumn id="6" name="Polistes L4 late vs early"/>
+    <tableColumn id="7" name="Polistes L5 late vs early"/>
+    <tableColumn id="8" name="Vespula L2 queen vs worker"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -691,12 +690,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>S7_Fig2A_regressions</t>
+          <t>S7_Fig2A_concordance</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Stagewise robust-regression results underlying Fig. 2A</t>
+          <t>Pairwise directional-concordance tests underlying Fig. 2A</t>
         </is>
       </c>
     </row>
@@ -708,12 +707,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>S8_Fig2B_ridge</t>
+          <t>S8_Fig2B_HOGs</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Nonnegative-ridge partial slopes underlying Fig. 2B</t>
+          <t>Functionally supported concordant HOGs displayed in Fig. 2B</t>
         </is>
       </c>
     </row>
@@ -4193,58 +4192,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Polistes_stage</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>HOGs</t>
+          <t>Vespula_stage</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Robust_slope</t>
+          <t>Jointly_DE_HOGs</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>Concordant_HOGs</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CI_95_lower</t>
+          <t>Concordant_fraction</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CI_95_upper</t>
+          <t>Expected_fraction_from_margins</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>P_value</t>
+          <t>Concordance_log2_odds_ratio</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Bonferroni_P</t>
+          <t>One_sided_Fisher_P</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>FDR_P_36_tests</t>
         </is>
       </c>
     </row>
@@ -4254,26 +4259,31 @@
           <t>L1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>0.004199923800915897</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>0.004274016388413369</v>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.004176994389708259</v>
+        <v>0.5957446808510638</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.01257684199154005</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>0.3257726314913849</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>1</v>
+        <v>0.4816659121774559</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1.398549376490275</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>0.09249823173385528</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>0.42797552836485</v>
       </c>
     </row>
     <row r="3">
@@ -4282,26 +4292,31 @@
           <t>L2</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.2161450851760437</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0.01419843779528823</v>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.1883166584605465</v>
+        <v>0.4</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.2439735118915409</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>2.482463358335303e-52</v>
+        <v>0.5111111111111111</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>-1.375170116164342</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1.489478015001182e-51</v>
+        <v>0.955422288855572</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -4310,26 +4325,31 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0.08742019022133553</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.009975721855564173</v>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.06786813466464067</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.1069722457780304</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>1.896251263621872e-18</v>
+        <v>0.4173553719008264</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>-1.473931188332412</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>1.137750758173123e-17</v>
+        <v>0.9464302467398442</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -4338,26 +4358,31 @@
           <t>L4</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>-0.04921212632260608</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>0.003277094432287645</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>11</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.0556351133838266</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.04278913926138556</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>5.682198724145955e-51</v>
+        <v>0.4955908289241622</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>-4.277360564261089</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>3.409319234487573e-50</v>
+        <v>0.9999999910193912</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4366,26 +4391,31 @@
           <t>L5</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>-0.3253767190460371</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0.02783261397398984</v>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>11</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>-0.3799276400306634</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-0.2708257980614108</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>1.425723533744882e-31</v>
+        <v>0.4104683195592286</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>-1.219507030292873</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>8.554341202469291e-31</v>
+        <v>0.9316833518724508</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -4394,30 +4424,1025 @@
           <t>P</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>1.183036072519082</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>0.03546841347056458</v>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1.113519259528</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>1.252552885510164</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>6.239859748096898e-244</v>
+        <v>0.5495867768595041</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.5703157247567547</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>3.743915848858139e-243</v>
+        <v>0.5103199174406604</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.7631578947368421</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.5155817174515236</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>3.251225103544161</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>8.295075542621677e-06</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>7.46556798835951e-05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.5084745762711864</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.4889399597816719</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.2246554728450171</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0.4845977663024635</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.3508771929824561</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.3379501385041551</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.1901028833799427</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.561228264890862</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.8208955223880597</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.5178213410559145</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>4.58408742030039</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>3.701040507470823e-14</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>6.661872913447482e-13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.8589743589743589</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.5013149243918474</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>5.090288885329103</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>6.510757451087585e-11</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>7.812908941305102e-10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.7251401587694165</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>0.3597620390789271</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0.9962641082185674</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.2962962962962963</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.3244170096021948</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>-0.7821763590616073</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.8543916007748462</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.4814814814814815</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>1.671898137492437</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0.09510567296996666</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.42797552836485</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.5185185185185185</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>1.765534746362977</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0.2013574660633485</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0.658988070752777</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.4997165532879818</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>-0.8081074623912335</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0.9363742493487888</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.4593195266272189</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>-1.04039458759356</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0.935541503277846</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.4866666666666667</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.1582620839167324</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>0.5955022488755624</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.4074074074074074</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.4567901234567901</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>-0.6539098544386477</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0.837916926704112</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>1.874469117916141</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>0.1674208144796379</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>0.6027149321266964</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.4545454545454546</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.5041322314049587</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>-0.4854268271702417</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0.8246753246753247</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0.5243055555555556</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>-0.5518202160985264</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>0.8335360894345217</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.4838709677419355</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.5171696149843913</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>-0.3992701834205273</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0.7823991230191356</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.380952380952381</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.4625850340136055</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>-1.17730453180791</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.9195046439628484</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.2568807339449541</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.4303088965575289</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>-2.655809899751786</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0.9999999993083226</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.3956834532374101</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.4871901040318824</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>-1.250110306611047</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>0.99454168554879</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.1836734693877551</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.5006247396917951</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>-4.248367627858496</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>0.999999999993858</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>394</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0.1852791878172589</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.5014687314798114</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>-4.415413849054691</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.3945945945945946</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.4962746530314098</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>-1.192496848234484</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>0.9983745637922488</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>81</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.5955882352941176</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0.5506055363321799</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0.7296422533603473</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>0.1460653677388139</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>0.5842614709552556</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.6506849315068494</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.5123850628635767</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>1.684296525653266</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>0.0005467214560014104</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>0.003936394483210154</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0.518796992481203</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0.4944880999491209</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0.3016556998611012</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>0.3429305995747384</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>0.9962641082185674</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.2337662337662338</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.4779895429246079</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>-3.633426756225302</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>0.9999997815060442</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>281</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>121</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0.4306049822064057</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0.4996517268018389</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>-0.7976652310048055</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>0.9926542321084004</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.6071428571428571</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.4946853741496599</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>1.450376460353516</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>0.00178689929713195</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0.0107213957827917</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>0.9473684210526316</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>0.5235457063711911</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>9.08695095847907</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>1.692645276844371e-40</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>6.093522996639736e-39</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4431,831 +5456,651 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vespula_response_stage</t>
+          <t>HOG</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Polistes_predictor_stage</t>
+          <t>Displayed_gene</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Stage_lag</t>
+          <t>Functional_group</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>HOGs</t>
+          <t>Selected_comparison</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Partial_slope</t>
+          <t>Polistes L1 late vs early</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Bootstrap_SE</t>
+          <t>Polistes L4 late vs early</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>CI_95_lower</t>
+          <t>Polistes L5 late vs early</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>CI_95_upper</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Centred_bootstrap_P</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Bonferroni_P</t>
+          <t>Vespula L2 queen vs worker</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0005758</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>0.007917829112406218</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>0.007467627810527557</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>0.02507760409252689</v>
-      </c>
-      <c r="I2" s="6" t="n">
-        <v>0.3173652694610778</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>1</v>
+          <t>Wdr59 (GATOR2)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>L1_to_L2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0.369 (*)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>-0.066 (ns)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>-0.055 (ns)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>0.523 (**)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0004507</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>1</v>
+          <t>nej/CBP</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>L1_to_L2</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>0.530 (*)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>0.427 (ns)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>0.065 (ns)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>0.508 (*)</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0008912</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>1</v>
+          <t>sut1-3 / SLC2-like</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-0.022 (ns)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0.942 (***)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0.060 (ns)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>0.605 (**)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0006185</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>-3</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>1</v>
+          <t>sgg/GSK3beta</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2; L5_to_L2</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>-0.081 (ns)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>0.631 (**)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>0.533 (**)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>0.666 (*)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0009263</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>-4</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>1</v>
+          <t>nmo/NLK</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>0.311 (ns)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>0.804 (*)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>0.170 (ns)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>0.688 (*)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>N13.HOG0010043</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>0.008160485569556298</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0.005119495399925694</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>3.913413379362141e-40</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.01881111009371601</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>0.1457085828343313</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>0.874251497005988</v>
+          <t>Gbs-76A</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>0.326 (ns)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>0.848 (*)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>0.259 (ns)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>0.416 (*)</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>N13.HOG0006961</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>0.1008162678804113</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0.01766517488059734</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>0.06675347708248081</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0.1354953690114516</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>0.001996007984031936</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>0.009980039920159681</v>
+          <t>Pepck</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>0.211 (ns)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1.332 (**)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>0.513 (ns)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>0.912 (*)</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>N13.HOG0007424</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0.03222681913591536</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.02669717918052739</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>0.09013243081129332</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>0.281437125748503</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>1</v>
+          <t>Pdk1</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>IIS/Wnt/mTOR/FoxO</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>-0.043 (ns)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>0.823 (*)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>0.081 (ns)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>0.925 (**)</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>N13.HOG0003585</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>0.09583408070110253</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0.01028823183972267</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>0.07572261547064263</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0.1140152979234217</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>0.001996007984031936</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>0.009980039920159681</v>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ecdysone/development</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>-0.133 (ns)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>0.766 (*)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>0.118 (ns)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>1.981 (***)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>N13.HOG0004754</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>-3</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>0.01093945972854783</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.01279200204541096</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>0.04230563548433951</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>0.4750499001996008</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>1</v>
+          <t>EcR</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Ecdysone/development</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>0.021 (ns)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>0.807 (*)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>0.085 (ns)</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>1.297 (***)</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>N13.HOG0005004</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>-4</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>0.01697168206193091</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0.00789275953758758</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>0.0008774147277418462</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>0.031858683321719</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>0.03592814371257485</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>0.1796407185628743</v>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Reproduction</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>0.325 (ns)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1.625 (**)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>0.164 (ns)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>1.140 (**)</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>N13.HOG0006201</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0.1098386797973152</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.01713364132481666</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>0.07690382871711894</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>0.1450477999730204</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>0.001996007984031936</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>0.007984031936127744</v>
+          <t>Actbeta</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Reproduction</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>0.125 (ns)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>1.856 (***)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>0.172 (ns)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>1.979 (**)</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>N13.HOG0000655</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1</v>
+          <t>bab1/2</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Reproduction</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>L5_to_L2</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>0.008 (ns)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1.594 (***)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1.737 (***)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>0.731 (*)</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>N13.HOG0006858</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>-2</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>-3</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>0.006664571147546513</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0.006932806661519308</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0.02429753682119604</v>
-      </c>
-      <c r="I16" s="6" t="n">
-        <v>0.4271457085828343</v>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>L4</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>-2</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>3.385222416752896e-42</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>L5</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>0.0005502886489110999</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>3.043700133333598e-41</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>5599</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>0.5838568770270605</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>0.0715955274198648</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>0.468576594708877</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>0.7466977823005572</v>
-      </c>
-      <c r="I22" s="6" t="n">
-        <v>0.001996007984031936</v>
-      </c>
-      <c r="J22" s="6" t="n">
-        <v>0.001996007984031936</v>
+          <t>Atg17</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Lifespan/diapause/stress</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>L4_to_L2</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>0.407 (ns)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>1.027 (**)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>0.366 (ns)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>0.591 (*)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J22"/>
+  <autoFilter ref="A1:H15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated PLS analysis table
</commit_message>
<xml_diff>
--- a/output/supplemental_tables/TablesS4-S8.xlsx
+++ b/output/supplemental_tables/TablesS4-S8.xlsx
@@ -9,20 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_DE_summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5A_PLS_axes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5B_PLS_LOOCV" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Fig1_GO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_Fig2A_concordance" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_Fig2B_HOGs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_PLS_LOOCV" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Fig1_GO" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_Fig2A_concordance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_Fig2B_HOGs" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table_index'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table_index'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'S4_DE_summary'!$A$1:$H$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S5A_PLS_axes'!$A$1:$E$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S5B_PLS_LOOCV'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S6_Fig1_GO'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S7_Fig2A_concordance'!$A$1:$I$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'S8_Fig2B_HOGs'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S5_PLS_LOOCV'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'S6_Fig1_GO'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S7_Fig2A_concordance'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S8_Fig2B_HOGs'!$A$1:$H$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -102,10 +100,10 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -188,8 +186,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SupplementaryTable1" displayName="SupplementaryTable1" ref="A1:C7" headerRowCount="1">
-  <autoFilter ref="A1:C7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SupplementaryTable1" displayName="SupplementaryTable1" ref="A1:C6" headerRowCount="1">
+  <autoFilter ref="A1:C6"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Table"/>
     <tableColumn id="2" name="Worksheet"/>
@@ -217,21 +215,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SupplementaryTable3" displayName="SupplementaryTable3" ref="A1:E4" headerRowCount="1">
-  <autoFilter ref="A1:E4"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Axis"/>
-    <tableColumn id="2" name="Biological_contrast"/>
-    <tableColumn id="3" name="PLS_component"/>
-    <tableColumn id="4" name="X_variance_explained_percent"/>
-    <tableColumn id="5" name="HOGs_in_final_model"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SupplementaryTable4" displayName="SupplementaryTable4" ref="A1:H13" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SupplementaryTable3" displayName="SupplementaryTable3" ref="A1:H13" headerRowCount="1">
   <autoFilter ref="A1:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Species"/>
@@ -241,14 +225,14 @@
     <tableColumn id="5" name="SE"/>
     <tableColumn id="6" name="df"/>
     <tableColumn id="7" name="t_ratio"/>
-    <tableColumn id="8" name="P_value"/>
+    <tableColumn id="8" name="One_sided_P"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SupplementaryTable5" displayName="SupplementaryTable5" ref="A1:I53" headerRowCount="1">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SupplementaryTable4" displayName="SupplementaryTable4" ref="A1:I53" headerRowCount="1">
   <autoFilter ref="A1:I53"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Category"/>
@@ -265,8 +249,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SupplementaryTable6" displayName="SupplementaryTable6" ref="A1:I37" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SupplementaryTable5" displayName="SupplementaryTable5" ref="A1:I37" headerRowCount="1">
   <autoFilter ref="A1:I37"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Polistes_stage"/>
@@ -283,8 +267,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SupplementaryTable7" displayName="SupplementaryTable7" ref="A1:H15" headerRowCount="1">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SupplementaryTable6" displayName="SupplementaryTable6" ref="A1:H15" headerRowCount="1">
   <autoFilter ref="A1:H15"/>
   <tableColumns count="8">
     <tableColumn id="1" name="HOG"/>
@@ -589,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -634,90 +618,73 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>S5A</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>S5A_PLS_axes</t>
+          <t>S5_PLS_LOOCV</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>PLS-axis mapping and variance explained</t>
+          <t>Planned one-sided season/caste contrasts from fully nested leave-one-sample-out PLS axis-1 scores</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S5B</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>S5B_PLS_LOOCV</t>
+          <t>S6_Fig1_GO</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Fully nested leave-one-sample-out season/caste contrasts on PLS axis 1</t>
+          <t>GO terms displayed in Fig. 1B</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>S6_Fig1_GO</t>
+          <t>S7_Fig2A_concordance</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>GO terms displayed in Fig. 1B</t>
+          <t>Pairwise directional-concordance tests underlying Fig. 2A</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>S7_Fig2A_concordance</t>
+          <t>S8_Fig2B_HOGs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Pairwise directional-concordance tests underlying Fig. 2A</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>S8</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>S8_Fig2B_HOGs</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
           <t>Functionally supported concordant HOGs displayed in Fig. 2B</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C7"/>
+  <autoFilter ref="A1:C6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1617,127 +1584,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Axis</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Biological_contrast</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>PLS_component</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>X_variance_explained_percent</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>HOGs_in_final_model</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Axis 1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Season/caste</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Component 3</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>8.246914618380515</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>4750</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Axis 2</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Developmental stage</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Component 2</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>22.24365449695813</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>4750</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Axis 3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Component 1</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>34.94062496076259</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>4750</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1789,7 +1635,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>P_value</t>
+          <t>One_sided_P</t>
         </is>
       </c>
     </row>
@@ -1821,8 +1667,8 @@
       <c r="G2" s="4" t="n">
         <v>3.734406432534832</v>
       </c>
-      <c r="H2" s="6" t="n">
-        <v>0.000285513773193567</v>
+      <c r="H2" s="5" t="n">
+        <v>0.0001427568865967835</v>
       </c>
     </row>
     <row r="3">
@@ -1841,20 +1687,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="6" t="n">
         <v>20.79307100651</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="6" t="n">
         <v>3.085264498191223</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="6" t="n">
         <v>6.739477610007251</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>5.33950840770262e-10</v>
+        <v>2.66975420385131e-10</v>
       </c>
     </row>
     <row r="4">
@@ -1885,8 +1731,8 @@
       <c r="G4" s="4" t="n">
         <v>4.431021233510832</v>
       </c>
-      <c r="H4" s="6" t="n">
-        <v>2.037539996101936e-05</v>
+      <c r="H4" s="5" t="n">
+        <v>1.018769998050968e-05</v>
       </c>
     </row>
     <row r="5">
@@ -1905,20 +1751,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="6" t="n">
         <v>18.43619661064062</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>2.712880600678148</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>6.795800967441052</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>4.018952358460656e-10</v>
+        <v>2.009476179230328e-10</v>
       </c>
     </row>
     <row r="6">
@@ -1949,8 +1795,8 @@
       <c r="G6" s="4" t="n">
         <v>3.742466874185742</v>
       </c>
-      <c r="H6" s="6" t="n">
-        <v>0.0002774118642823559</v>
+      <c r="H6" s="5" t="n">
+        <v>0.000138705932141178</v>
       </c>
     </row>
     <row r="7">
@@ -1969,20 +1815,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="6" t="n">
         <v>18.83256735309037</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <v>3.91695192785582</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="6" t="n">
         <v>4.807964892078598</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>4.330032794783674e-06</v>
+        <v>2.165016397391837e-06</v>
       </c>
     </row>
     <row r="8">
@@ -2013,8 +1859,8 @@
       <c r="G8" s="4" t="n">
         <v>1.979880915018535</v>
       </c>
-      <c r="H8" s="6" t="n">
-        <v>0.04993156740734814</v>
+      <c r="H8" s="5" t="n">
+        <v>0.02496578370367407</v>
       </c>
     </row>
     <row r="9">
@@ -2033,20 +1879,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="6" t="n">
         <v>12.46997147942485</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <v>2.56215751257896</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="6" t="n">
         <v>4.866980823077151</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>3.373699424199353e-06</v>
+        <v>1.686849712099677e-06</v>
       </c>
     </row>
     <row r="10">
@@ -2077,8 +1923,8 @@
       <c r="G10" s="4" t="n">
         <v>2.342503166538906</v>
       </c>
-      <c r="H10" s="6" t="n">
-        <v>0.02074789490369007</v>
+      <c r="H10" s="5" t="n">
+        <v>0.01037394745184503</v>
       </c>
     </row>
     <row r="11">
@@ -2097,20 +1943,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="6" t="n">
         <v>10.11309708355547</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="6" t="n">
         <v>2.818300253034161</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <v>3.58836751785683</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.0004774112019446483</v>
+        <v>0.0002387056009723242</v>
       </c>
     </row>
     <row r="12">
@@ -2141,8 +1987,8 @@
       <c r="G12" s="4" t="n">
         <v>1.571205351258403</v>
       </c>
-      <c r="H12" s="6" t="n">
-        <v>0.1186831866705417</v>
+      <c r="H12" s="5" t="n">
+        <v>0.05934159333527084</v>
       </c>
     </row>
     <row r="13">
@@ -2161,20 +2007,20 @@
           <t>(L/Q) - (E/W)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="6" t="n">
         <v>10.50946782600522</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="6" t="n">
         <v>3.577878784298491</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <v>2.937345969384424</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.003947758446536406</v>
+        <v>0.001973879223268203</v>
       </c>
     </row>
   </sheetData>
@@ -2186,7 +2032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2281,7 +2127,7 @@
       <c r="G2" s="4" t="n">
         <v>6.914893617021277</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="5" t="n">
         <v>5.1e-09</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2312,10 +2158,10 @@
       <c r="E3" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6" t="n">
         <v>16.58</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="6" t="n">
         <v>2.714113389626056</v>
       </c>
       <c r="H3" s="7" t="n">
@@ -2355,7 +2201,7 @@
       <c r="G4" s="4" t="n">
         <v>6.206896551724138</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>4e-06</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2386,10 +2232,10 @@
       <c r="E5" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>3.19</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>4.075235109717869</v>
       </c>
       <c r="H5" s="7" t="n">
@@ -2429,7 +2275,7 @@
       <c r="G6" s="4" t="n">
         <v>4.926108374384237</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="5" t="n">
         <v>1.4e-05</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2460,10 +2306,10 @@
       <c r="E7" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="6" t="n">
         <v>2.97</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="6" t="n">
         <v>4.04040404040404</v>
       </c>
       <c r="H7" s="7" t="n">
@@ -2503,7 +2349,7 @@
       <c r="G8" s="4" t="n">
         <v>4.761904761904762</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="5" t="n">
         <v>2e-05</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -2534,10 +2380,10 @@
       <c r="E9" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <v>16.51</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="6" t="n">
         <v>2.483343428225318</v>
       </c>
       <c r="H9" s="7" t="n">
@@ -2577,7 +2423,7 @@
       <c r="G10" s="4" t="n">
         <v>4.972375690607735</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="5" t="n">
         <v>3.5e-05</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -2608,10 +2454,10 @@
       <c r="E11" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <v>1.52</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <v>5.263157894736842</v>
       </c>
       <c r="H11" s="7" t="n">
@@ -2651,7 +2497,7 @@
       <c r="G12" s="4" t="n">
         <v>5.723905723905723</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>0.00011</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2682,10 +2528,10 @@
       <c r="E13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <v>3.48</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <v>3.448275862068966</v>
       </c>
       <c r="H13" s="7" t="n">
@@ -2725,7 +2571,7 @@
       <c r="G14" s="4" t="n">
         <v>4.790419161676647</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="5" t="n">
         <v>0.00013</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -2756,10 +2602,10 @@
       <c r="E15" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <v>4.285714285714286</v>
       </c>
       <c r="H15" s="7" t="n">
@@ -2799,7 +2645,7 @@
       <c r="G16" s="4" t="n">
         <v>3.201970443349754</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="5" t="n">
         <v>0.00013</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2830,10 +2676,10 @@
       <c r="E17" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="6" t="n">
         <v>14.41</v>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="6" t="n">
         <v>2.290076335877862</v>
       </c>
       <c r="H17" s="7" t="n">
@@ -2873,7 +2719,7 @@
       <c r="G18" s="4" t="n">
         <v>3.568075117370892</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="5" t="n">
         <v>0.00037</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -2904,10 +2750,10 @@
       <c r="E19" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="6" t="n">
         <v>7.39</v>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="6" t="n">
         <v>3.788903924221922</v>
       </c>
       <c r="H19" s="7" t="n">
@@ -2947,7 +2793,7 @@
       <c r="G20" s="4" t="n">
         <v>4.605263157894737</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H20" s="5" t="n">
         <v>0.00047</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2978,10 +2824,10 @@
       <c r="E21" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>2.46</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="6" t="n">
         <v>3.658536585365854</v>
       </c>
       <c r="H21" s="7" t="n">
@@ -3021,7 +2867,7 @@
       <c r="G22" s="4" t="n">
         <v>3.367003367003367</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="5" t="n">
         <v>0.0005</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -3052,10 +2898,10 @@
       <c r="E23" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="6" t="n">
         <v>2.03</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="6" t="n">
         <v>3.94088669950739</v>
       </c>
       <c r="H23" s="7" t="n">
@@ -3095,7 +2941,7 @@
       <c r="G24" s="4" t="n">
         <v>3.034901365705615</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="5" t="n">
         <v>0.00082</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -3126,10 +2972,10 @@
       <c r="E25" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="6" t="n">
         <v>2.75</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="6" t="n">
         <v>3.272727272727273</v>
       </c>
       <c r="H25" s="7" t="n">
@@ -3169,7 +3015,7 @@
       <c r="G26" s="4" t="n">
         <v>3.571428571428571</v>
       </c>
-      <c r="H26" s="6" t="n">
+      <c r="H26" s="5" t="n">
         <v>0.00124</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -3200,10 +3046,10 @@
       <c r="E27" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="6" t="n">
         <v>2.39</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="6" t="n">
         <v>3.765690376569037</v>
       </c>
       <c r="H27" s="7" t="n">
@@ -3243,7 +3089,7 @@
       <c r="G28" s="4" t="n">
         <v>4.825291181364393</v>
       </c>
-      <c r="H28" s="6" t="n">
+      <c r="H28" s="5" t="n">
         <v>0.00193</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -3274,10 +3120,10 @@
       <c r="E29" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="6" t="n">
         <v>8.26</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="6" t="n">
         <v>1.573849878934625</v>
       </c>
       <c r="H29" s="7" t="n">
@@ -3317,7 +3163,7 @@
       <c r="G30" s="4" t="n">
         <v>3.252032520325203</v>
       </c>
-      <c r="H30" s="6" t="n">
+      <c r="H30" s="5" t="n">
         <v>0.00236</v>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3348,10 +3194,10 @@
       <c r="E31" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="6" t="n">
         <v>2.1</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="6" t="n">
         <v>3.333333333333333</v>
       </c>
       <c r="H31" s="7" t="n">
@@ -3391,7 +3237,7 @@
       <c r="G32" s="4" t="n">
         <v>3.333333333333333</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="5" t="n">
         <v>0.00378</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3422,10 +3268,10 @@
       <c r="E33" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="6" t="n">
         <v>9.99</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="6" t="n">
         <v>2.302302302302302</v>
       </c>
       <c r="H33" s="7" t="n">
@@ -3465,7 +3311,7 @@
       <c r="G34" s="4" t="n">
         <v>3.618421052631579</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H34" s="5" t="n">
         <v>0.00013</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3496,10 +3342,10 @@
       <c r="E35" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="6" t="n">
         <v>8.69</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="6" t="n">
         <v>1.956271576524741</v>
       </c>
       <c r="H35" s="7" t="n">
@@ -3539,7 +3385,7 @@
       <c r="G36" s="4" t="n">
         <v>3.252032520325203</v>
       </c>
-      <c r="H36" s="6" t="n">
+      <c r="H36" s="5" t="n">
         <v>0.00236</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -3570,10 +3416,10 @@
       <c r="E37" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="6" t="n">
         <v>12.17</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="6" t="n">
         <v>1.725554642563681</v>
       </c>
       <c r="H37" s="7" t="n">
@@ -3613,7 +3459,7 @@
       <c r="G38" s="4" t="n">
         <v>4.137931034482759</v>
       </c>
-      <c r="H38" s="6" t="n">
+      <c r="H38" s="5" t="n">
         <v>0.00222</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -3644,10 +3490,10 @@
       <c r="E39" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="6" t="n">
         <v>2.75</v>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="6" t="n">
         <v>2.545454545454545</v>
       </c>
       <c r="H39" s="7" t="n">
@@ -3687,7 +3533,7 @@
       <c r="G40" s="4" t="n">
         <v>2.955665024630542</v>
       </c>
-      <c r="H40" s="6" t="n">
+      <c r="H40" s="5" t="n">
         <v>0.01324</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3718,10 +3564,10 @@
       <c r="E41" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="6" t="n">
         <v>2.61</v>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="6" t="n">
         <v>5.363984674329502</v>
       </c>
       <c r="H41" s="7" t="n">
@@ -3761,7 +3607,7 @@
       <c r="G42" s="4" t="n">
         <v>3.236797274275979</v>
       </c>
-      <c r="H42" s="6" t="n">
+      <c r="H42" s="5" t="n">
         <v>3e-06</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3792,10 +3638,10 @@
       <c r="E43" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="F43" s="5" t="n">
+      <c r="F43" s="6" t="n">
         <v>18.1</v>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="6" t="n">
         <v>2.265193370165746</v>
       </c>
       <c r="H43" s="7" t="n">
@@ -3835,7 +3681,7 @@
       <c r="G44" s="4" t="n">
         <v>2.412868632707775</v>
       </c>
-      <c r="H44" s="6" t="n">
+      <c r="H44" s="5" t="n">
         <v>0.00014</v>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -3866,10 +3712,10 @@
       <c r="E45" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="6" t="n">
         <v>3.125</v>
       </c>
       <c r="H45" s="7" t="n">
@@ -3909,7 +3755,7 @@
       <c r="G46" s="4" t="n">
         <v>3.067484662576687</v>
       </c>
-      <c r="H46" s="6" t="n">
+      <c r="H46" s="5" t="n">
         <v>0.00111</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3940,10 +3786,10 @@
       <c r="E47" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="6" t="n">
         <v>1.74</v>
       </c>
-      <c r="G47" s="5" t="n">
+      <c r="G47" s="6" t="n">
         <v>4.022988505747127</v>
       </c>
       <c r="H47" s="7" t="n">
@@ -3983,7 +3829,7 @@
       <c r="G48" s="4" t="n">
         <v>1.865671641791045</v>
       </c>
-      <c r="H48" s="6" t="n">
+      <c r="H48" s="5" t="n">
         <v>0.00124</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -4014,10 +3860,10 @@
       <c r="E49" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="6" t="n">
         <v>1.45</v>
       </c>
-      <c r="G49" s="5" t="n">
+      <c r="G49" s="6" t="n">
         <v>4.137931034482759</v>
       </c>
       <c r="H49" s="7" t="n">
@@ -4057,7 +3903,7 @@
       <c r="G50" s="4" t="n">
         <v>2.155172413793104</v>
       </c>
-      <c r="H50" s="6" t="n">
+      <c r="H50" s="5" t="n">
         <v>0.00256</v>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -4088,10 +3934,10 @@
       <c r="E51" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="6" t="n">
         <v>4.63</v>
       </c>
-      <c r="G51" s="5" t="n">
+      <c r="G51" s="6" t="n">
         <v>2.375809935205184</v>
       </c>
       <c r="H51" s="7" t="n">
@@ -4131,7 +3977,7 @@
       <c r="G52" s="4" t="n">
         <v>2.576112412177986</v>
       </c>
-      <c r="H52" s="6" t="n">
+      <c r="H52" s="5" t="n">
         <v>0.00287</v>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -4162,10 +4008,10 @@
       <c r="E53" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="6" t="n">
         <v>1.52</v>
       </c>
-      <c r="G53" s="5" t="n">
+      <c r="G53" s="6" t="n">
         <v>3.947368421052631</v>
       </c>
       <c r="H53" s="7" t="n">
@@ -4186,7 +4032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4279,10 +4125,10 @@
       <c r="G2" s="4" t="n">
         <v>1.398549376490275</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="5" t="n">
         <v>0.09249823173385528</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="5" t="n">
         <v>0.42797552836485</v>
       </c>
     </row>
@@ -4303,17 +4149,17 @@
       <c r="D3" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6" t="n">
         <v>0.5111111111111111</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="6" t="n">
         <v>-1.375170116164342</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.955422288855572</v>
+        <v>0.9554222888555721</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>1</v>
@@ -4345,7 +4191,7 @@
       <c r="G4" s="4" t="n">
         <v>-1.473931188332412</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.9464302467398442</v>
       </c>
       <c r="I4" s="2" t="n">
@@ -4369,17 +4215,17 @@
       <c r="D5" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>0.1746031746031746</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>0.4955908289241622</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>-4.277360564261089</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.9999999910193912</v>
+        <v>0.9999999910193911</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>1</v>
@@ -4411,8 +4257,8 @@
       <c r="G6" s="4" t="n">
         <v>-1.219507030292873</v>
       </c>
-      <c r="H6" s="6" t="n">
-        <v>0.9316833518724508</v>
+      <c r="H6" s="5" t="n">
+        <v>0.9316833518724509</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
@@ -4435,13 +4281,13 @@
       <c r="D7" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <v>0.5909090909090909</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="6" t="n">
         <v>0.5495867768595041</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="6" t="n">
         <v>0.5703157247567547</v>
       </c>
       <c r="H7" s="7" t="n">
@@ -4477,10 +4323,10 @@
       <c r="G8" s="4" t="n">
         <v>3.251225103544161</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="5" t="n">
         <v>8.295075542621677e-06</v>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I8" s="5" t="n">
         <v>7.46556798835951e-05</v>
       </c>
     </row>
@@ -4501,14 +4347,14 @@
       <c r="D9" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <v>0.5084745762711864</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <v>0.4889399597816719</v>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>0.2246554728450171</v>
+      <c r="G9" s="6" t="n">
+        <v>0.224655472845017</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>0.4845977663024635</v>
@@ -4543,7 +4389,7 @@
       <c r="G10" s="4" t="n">
         <v>0.1901028833799427</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="5" t="n">
         <v>0.561228264890862</v>
       </c>
       <c r="I10" s="2" t="n">
@@ -4567,20 +4413,20 @@
       <c r="D11" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="6" t="n">
         <v>0.8208955223880597</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <v>0.5178213410559145</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <v>4.58408742030039</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>3.701040507470823e-14</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>6.661872913447482e-13</v>
+        <v>6.661872913447481e-13</v>
       </c>
     </row>
     <row r="12">
@@ -4609,10 +4455,10 @@
       <c r="G12" s="4" t="n">
         <v>5.090288885329103</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>6.510757451087585e-11</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="5" t="n">
         <v>7.812908941305102e-10</v>
       </c>
     </row>
@@ -4633,13 +4479,13 @@
       <c r="D13" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <v>0.45</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <v>0.7251401587694165</v>
       </c>
       <c r="H13" s="7" t="n">
@@ -4675,7 +4521,7 @@
       <c r="G14" s="4" t="n">
         <v>-0.7821763590616073</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="5" t="n">
         <v>0.8543916007748462</v>
       </c>
       <c r="I14" s="2" t="n">
@@ -4699,13 +4545,13 @@
       <c r="D15" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>0.6111111111111112</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <v>0.4814814814814815</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <v>1.671898137492437</v>
       </c>
       <c r="H15" s="7" t="n">
@@ -4741,10 +4587,10 @@
       <c r="G16" s="4" t="n">
         <v>1.765534746362977</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="5" t="n">
         <v>0.2013574660633485</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="5" t="n">
         <v>0.658988070752777</v>
       </c>
     </row>
@@ -4765,13 +4611,13 @@
       <c r="D17" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="6" t="n">
         <v>0.4285714285714285</v>
       </c>
-      <c r="F17" s="5" t="n">
-        <v>0.4997165532879818</v>
-      </c>
-      <c r="G17" s="5" t="n">
+      <c r="F17" s="6" t="n">
+        <v>0.4997165532879819</v>
+      </c>
+      <c r="G17" s="6" t="n">
         <v>-0.8081074623912335</v>
       </c>
       <c r="H17" s="7" t="n">
@@ -4805,9 +4651,9 @@
         <v>0.4593195266272189</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>-1.04039458759356</v>
-      </c>
-      <c r="H18" s="6" t="n">
+        <v>-1.040394587593561</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>0.935541503277846</v>
       </c>
       <c r="I18" s="2" t="n">
@@ -4831,13 +4677,13 @@
       <c r="D19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="6" t="n">
         <v>0.4866666666666667</v>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="6" t="n">
         <v>0.1582620839167324</v>
       </c>
       <c r="H19" s="7" t="n">
@@ -4873,7 +4719,7 @@
       <c r="G20" s="4" t="n">
         <v>-0.6539098544386477</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H20" s="5" t="n">
         <v>0.837916926704112</v>
       </c>
       <c r="I20" s="2" t="n">
@@ -4897,13 +4743,13 @@
       <c r="D21" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="6" t="n">
         <v>1.874469117916141</v>
       </c>
       <c r="H21" s="7" t="n">
@@ -4931,7 +4777,7 @@
         <v>5</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.4545454545454546</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>0.5041322314049587</v>
@@ -4939,7 +4785,7 @@
       <c r="G22" s="4" t="n">
         <v>-0.4854268271702417</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="5" t="n">
         <v>0.8246753246753247</v>
       </c>
       <c r="I22" s="2" t="n">
@@ -4963,13 +4809,13 @@
       <c r="D23" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="6" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="6" t="n">
         <v>0.5243055555555556</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="6" t="n">
         <v>-0.5518202160985264</v>
       </c>
       <c r="H23" s="7" t="n">
@@ -5005,7 +4851,7 @@
       <c r="G24" s="4" t="n">
         <v>-0.3992701834205273</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="5" t="n">
         <v>0.7823991230191356</v>
       </c>
       <c r="I24" s="2" t="n">
@@ -5029,17 +4875,17 @@
       <c r="D25" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="E25" s="5" t="n">
-        <v>0.380952380952381</v>
-      </c>
-      <c r="F25" s="5" t="n">
+      <c r="E25" s="6" t="n">
+        <v>0.3809523809523809</v>
+      </c>
+      <c r="F25" s="6" t="n">
         <v>0.4625850340136055</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="6" t="n">
         <v>-1.17730453180791</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.9195046439628484</v>
+        <v>0.9195046439628483</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1</v>
@@ -5071,7 +4917,7 @@
       <c r="G26" s="4" t="n">
         <v>-2.655809899751786</v>
       </c>
-      <c r="H26" s="6" t="n">
+      <c r="H26" s="5" t="n">
         <v>0.9999999993083226</v>
       </c>
       <c r="I26" s="2" t="n">
@@ -5095,13 +4941,13 @@
       <c r="D27" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="6" t="n">
         <v>0.3956834532374101</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="6" t="n">
         <v>0.4871901040318824</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="6" t="n">
         <v>-1.250110306611047</v>
       </c>
       <c r="H27" s="7" t="n">
@@ -5137,7 +4983,7 @@
       <c r="G28" s="4" t="n">
         <v>-4.248367627858496</v>
       </c>
-      <c r="H28" s="6" t="n">
+      <c r="H28" s="5" t="n">
         <v>0.999999999993858</v>
       </c>
       <c r="I28" s="2" t="n">
@@ -5161,13 +5007,13 @@
       <c r="D29" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="6" t="n">
         <v>0.1852791878172589</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="6" t="n">
         <v>0.5014687314798114</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="6" t="n">
         <v>-4.415413849054691</v>
       </c>
       <c r="H29" s="3" t="n">
@@ -5203,7 +5049,7 @@
       <c r="G30" s="4" t="n">
         <v>-1.192496848234484</v>
       </c>
-      <c r="H30" s="6" t="n">
+      <c r="H30" s="5" t="n">
         <v>0.9983745637922488</v>
       </c>
       <c r="I30" s="2" t="n">
@@ -5227,13 +5073,13 @@
       <c r="D31" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="6" t="n">
         <v>0.5955882352941176</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="6" t="n">
         <v>0.5506055363321799</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="6" t="n">
         <v>0.7296422533603473</v>
       </c>
       <c r="H31" s="7" t="n">
@@ -5269,10 +5115,10 @@
       <c r="G32" s="4" t="n">
         <v>1.684296525653266</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="5" t="n">
         <v>0.0005467214560014104</v>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="I32" s="5" t="n">
         <v>0.003936394483210154</v>
       </c>
     </row>
@@ -5293,13 +5139,13 @@
       <c r="D33" s="3" t="n">
         <v>69</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E33" s="6" t="n">
         <v>0.518796992481203</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="6" t="n">
         <v>0.4944880999491209</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="6" t="n">
         <v>0.3016556998611012</v>
       </c>
       <c r="H33" s="7" t="n">
@@ -5335,7 +5181,7 @@
       <c r="G34" s="4" t="n">
         <v>-3.633426756225302</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H34" s="5" t="n">
         <v>0.9999997815060442</v>
       </c>
       <c r="I34" s="2" t="n">
@@ -5359,17 +5205,17 @@
       <c r="D35" s="3" t="n">
         <v>121</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="6" t="n">
         <v>0.4306049822064057</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="6" t="n">
         <v>0.4996517268018389</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="6" t="n">
         <v>-0.7976652310048055</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.9926542321084004</v>
+        <v>0.9926542321084005</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>1</v>
@@ -5401,11 +5247,11 @@
       <c r="G36" s="4" t="n">
         <v>1.450376460353516</v>
       </c>
-      <c r="H36" s="6" t="n">
-        <v>0.00178689929713195</v>
-      </c>
-      <c r="I36" s="6" t="n">
-        <v>0.0107213957827917</v>
+      <c r="H36" s="5" t="n">
+        <v>0.001786899297131958</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>0.01072139578279175</v>
       </c>
     </row>
     <row r="37">
@@ -5425,20 +5271,20 @@
       <c r="D37" s="3" t="n">
         <v>180</v>
       </c>
-      <c r="E37" s="5" t="n">
-        <v>0.9473684210526316</v>
-      </c>
-      <c r="F37" s="5" t="n">
+      <c r="E37" s="6" t="n">
+        <v>0.9473684210526315</v>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>0.5235457063711911</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="6" t="n">
         <v>9.08695095847907</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>1.692645276844371e-40</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>6.093522996639736e-39</v>
+        <v>6.093522996639737e-39</v>
       </c>
     </row>
   </sheetData>
@@ -5450,7 +5296,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5514,12 +5360,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0005758</t>
+          <t>N13.HOG0010043</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Wdr59 (GATOR2)</t>
+          <t>Gbs-76A</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -5529,39 +5375,39 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>L1_to_L2</t>
+          <t>L4_to_L2</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0.369 (*)</t>
+          <t>0.326 (ns)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>-0.066 (ns)</t>
+          <t>0.848 (*)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>-0.055 (ns)</t>
+          <t>0.259 (ns)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>0.523 (**)</t>
+          <t>0.416 (*)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0004507</t>
+          <t>N13.HOG0007424</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>nej/CBP</t>
+          <t>Pdk1</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -5571,39 +5417,39 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>L1_to_L2</t>
+          <t>L4_to_L2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>0.530 (*)</t>
+          <t>-0.043 (ns)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>0.427 (ns)</t>
+          <t>0.823 (*)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>0.065 (ns)</t>
+          <t>0.081 (ns)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>0.508 (*)</t>
+          <t>0.925 (**)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0008912</t>
+          <t>N13.HOG0006961</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sut1-3 / SLC2-like</t>
+          <t>Pepck</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -5618,34 +5464,34 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>-0.022 (ns)</t>
+          <t>0.211 (ns)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>0.942 (***)</t>
+          <t>1.332 (**)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.060 (ns)</t>
+          <t>0.513 (ns)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>0.605 (**)</t>
+          <t>0.912 (*)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0006185</t>
+          <t>N13.HOG0005758</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>sgg/GSK3beta</t>
+          <t>Wdr59 (GATOR2)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -5655,39 +5501,39 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>L4_to_L2; L5_to_L2</t>
+          <t>L1_to_L2</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>-0.081 (ns)</t>
+          <t>0.369 (*)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>0.631 (**)</t>
+          <t>-0.066 (ns)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>0.533 (**)</t>
+          <t>-0.055 (ns)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>0.666 (*)</t>
+          <t>0.523 (**)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0009263</t>
+          <t>N13.HOG0004507</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>nmo/NLK</t>
+          <t>nej/CBP</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -5697,39 +5543,39 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>L4_to_L2</t>
+          <t>L1_to_L2</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.311 (ns)</t>
+          <t>0.530 (*)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>0.804 (*)</t>
+          <t>0.427 (ns)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.170 (ns)</t>
+          <t>0.065 (ns)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>0.688 (*)</t>
+          <t>0.508 (*)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0010043</t>
+          <t>N13.HOG0009263</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Gbs-76A</t>
+          <t>nmo/NLK</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -5744,34 +5590,34 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>0.326 (ns)</t>
+          <t>0.311 (ns)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>0.848 (*)</t>
+          <t>0.804 (*)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>0.259 (ns)</t>
+          <t>0.170 (ns)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>0.416 (*)</t>
+          <t>0.688 (*)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0006961</t>
+          <t>N13.HOG0006185</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Pepck</t>
+          <t>sgg/GSK3beta</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -5781,39 +5627,39 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>L4_to_L2</t>
+          <t>L4_to_L2; L5_to_L2</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0.211 (ns)</t>
+          <t>-0.081 (ns)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1.332 (**)</t>
+          <t>0.631 (**)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.513 (ns)</t>
+          <t>0.533 (**)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>0.912 (*)</t>
+          <t>0.666 (*)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0007424</t>
+          <t>N13.HOG0008912</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Pdk1</t>
+          <t>sut1-3 / SLC2-like</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -5828,34 +5674,34 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-0.043 (ns)</t>
+          <t>-0.022 (ns)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>0.823 (*)</t>
+          <t>0.942 (***)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>0.081 (ns)</t>
+          <t>0.060 (ns)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>0.925 (**)</t>
+          <t>0.605 (**)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0003585</t>
+          <t>N13.HOG0004754</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>br</t>
+          <t>EcR</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -5870,34 +5716,34 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>-0.133 (ns)</t>
+          <t>0.021 (ns)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>0.766 (*)</t>
+          <t>0.807 (*)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.118 (ns)</t>
+          <t>0.085 (ns)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>1.981 (***)</t>
+          <t>1.297 (***)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0004754</t>
+          <t>N13.HOG0003585</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>EcR</t>
+          <t>br</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -5912,34 +5758,34 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>0.021 (ns)</t>
+          <t>-0.133 (ns)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>0.807 (*)</t>
+          <t>0.766 (*)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>0.085 (ns)</t>
+          <t>0.118 (ns)</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>1.297 (***)</t>
+          <t>1.981 (***)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0005004</t>
+          <t>N13.HOG0006201</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>Actbeta</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -5954,34 +5800,34 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0.325 (ns)</t>
+          <t>0.125 (ns)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1.625 (**)</t>
+          <t>1.856 (***)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.164 (ns)</t>
+          <t>0.172 (ns)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>1.140 (**)</t>
+          <t>1.979 (**)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>N13.HOG0006201</t>
+          <t>N13.HOG0000655</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Actbeta</t>
+          <t>bab1/2</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -5991,39 +5837,39 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>L4_to_L2</t>
+          <t>L5_to_L2</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>0.125 (ns)</t>
+          <t>0.008 (ns)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>1.856 (***)</t>
+          <t>1.594 (***)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>0.172 (ns)</t>
+          <t>1.737 (***)</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>1.979 (**)</t>
+          <t>0.731 (*)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>N13.HOG0000655</t>
+          <t>N13.HOG0005004</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>bab1/2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6033,27 +5879,27 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>L5_to_L2</t>
+          <t>L4_to_L2</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>0.008 (ns)</t>
+          <t>0.325 (ns)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1.594 (***)</t>
+          <t>1.625 (**)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1.737 (***)</t>
+          <t>0.164 (ns)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>0.731 (*)</t>
+          <t>1.140 (**)</t>
         </is>
       </c>
     </row>

</xml_diff>